<commit_message>
chore(data): batch update intraday dim_rca - 11:51:28
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2584"/>
+  <dimension ref="A1:D2585"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44725,7 +44725,7 @@
       </c>
       <c r="C2461" t="inlineStr">
         <is>
-          <t>CAROLINE L. DA HORA - FARMA (SSA CENTRO)</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2461" t="n">
@@ -45185,37 +45185,37 @@
     <row r="2487">
       <c r="A2487" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2487" t="n">
-        <v>2792</v>
+        <v>2823</v>
       </c>
       <c r="C2487" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2487" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2488">
       <c r="A2488" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2488" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2488" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2488" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2489">
@@ -45225,15 +45225,15 @@
         </is>
       </c>
       <c r="B2489" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2489" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2489" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2490">
@@ -45243,15 +45243,15 @@
         </is>
       </c>
       <c r="B2490" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2490" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2490" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2491">
@@ -45261,15 +45261,15 @@
         </is>
       </c>
       <c r="B2491" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2491" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2491" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2492">
@@ -45279,11 +45279,11 @@
         </is>
       </c>
       <c r="B2492" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2492" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D2492" t="n">
@@ -45293,37 +45293,37 @@
     <row r="2493">
       <c r="A2493" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2493" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2493" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2493" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2494">
       <c r="A2494" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2494" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2494" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2494" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2495">
@@ -45333,11 +45333,11 @@
         </is>
       </c>
       <c r="B2495" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2495" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2495" t="n">
@@ -45347,55 +45347,55 @@
     <row r="2496">
       <c r="A2496" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2496" t="n">
-        <v>2642</v>
+        <v>2769</v>
       </c>
       <c r="C2496" t="inlineStr">
         <is>
-          <t>H-VAGO DESIREE BARROS DE CARVALHO</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2496" t="n">
-        <v>52</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2497">
       <c r="A2497" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2497" t="n">
-        <v>2649</v>
+        <v>2642</v>
       </c>
       <c r="C2497" t="inlineStr">
         <is>
-          <t>HERTZ PE - (VAGO/DIEGO CALABRIA)</t>
+          <t>H-VAGO DESIREE BARROS DE CARVALHO</t>
         </is>
       </c>
       <c r="D2497" t="n">
-        <v>142</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2498">
       <c r="A2498" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2498" t="n">
-        <v>2679</v>
+        <v>2649</v>
       </c>
       <c r="C2498" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>HERTZ PE - (VAGO/DIEGO CALABRIA)</t>
         </is>
       </c>
       <c r="D2498" t="n">
-        <v>69</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2499">
@@ -45405,11 +45405,11 @@
         </is>
       </c>
       <c r="B2499" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2499" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2499" t="n">
@@ -45419,19 +45419,19 @@
     <row r="2500">
       <c r="A2500" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2500" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2500" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2500" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2501">
@@ -45441,15 +45441,15 @@
         </is>
       </c>
       <c r="B2501" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2501" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2501" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2502">
@@ -45459,11 +45459,11 @@
         </is>
       </c>
       <c r="B2502" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2502" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2502" t="n">
@@ -45473,37 +45473,37 @@
     <row r="2503">
       <c r="A2503" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2503" t="n">
-        <v>2701</v>
+        <v>2817</v>
       </c>
       <c r="C2503" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2503" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2504">
       <c r="A2504" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2504" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2504" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2504" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2505">
@@ -45513,11 +45513,11 @@
         </is>
       </c>
       <c r="B2505" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2505" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2505" t="n">
@@ -45527,19 +45527,19 @@
     <row r="2506">
       <c r="A2506" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B2506" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2506" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2506" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2507">
@@ -45549,51 +45549,51 @@
         </is>
       </c>
       <c r="B2507" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2507" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2507" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2508">
       <c r="A2508" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2508" t="n">
-        <v>2788</v>
+        <v>2755</v>
       </c>
       <c r="C2508" t="inlineStr">
         <is>
-          <t>H-ARTHUR GV HERTZ</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2508" t="n">
-        <v>52</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2509">
       <c r="A2509" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2509" t="n">
-        <v>2665</v>
+        <v>2788</v>
       </c>
       <c r="C2509" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>H-ARTHUR GV HERTZ</t>
         </is>
       </c>
       <c r="D2509" t="n">
-        <v>141</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2510">
@@ -45603,15 +45603,15 @@
         </is>
       </c>
       <c r="B2510" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2510" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2510" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2511">
@@ -45621,15 +45621,15 @@
         </is>
       </c>
       <c r="B2511" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2511" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
         </is>
       </c>
       <c r="D2511" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2512">
@@ -45639,11 +45639,11 @@
         </is>
       </c>
       <c r="B2512" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2512" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2512" t="n">
@@ -45653,37 +45653,37 @@
     <row r="2513">
       <c r="A2513" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2513" t="n">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="C2513" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2513" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2514">
       <c r="A2514" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2514" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2514" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2514" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2515">
@@ -45693,11 +45693,11 @@
         </is>
       </c>
       <c r="B2515" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2515" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2515" t="n">
@@ -45711,15 +45711,15 @@
         </is>
       </c>
       <c r="B2516" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2516" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2516" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2517">
@@ -45729,11 +45729,11 @@
         </is>
       </c>
       <c r="B2517" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2517" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - HB</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2517" t="n">
@@ -45747,15 +45747,15 @@
         </is>
       </c>
       <c r="B2518" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2518" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - HB</t>
         </is>
       </c>
       <c r="D2518" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2519">
@@ -45765,51 +45765,51 @@
         </is>
       </c>
       <c r="B2519" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2519" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2519" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2520">
       <c r="A2520" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2520" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2520" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2520" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2521">
       <c r="A2521" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2521" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2521" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2521" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2522">
@@ -45819,33 +45819,33 @@
         </is>
       </c>
       <c r="B2522" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2522" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2522" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2523">
       <c r="A2523" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2523" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2523" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2523" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2524">
@@ -45855,69 +45855,69 @@
         </is>
       </c>
       <c r="B2524" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2524" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2524" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2525">
       <c r="A2525" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2525" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2525" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2525" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2526">
       <c r="A2526" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2526" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2526" t="inlineStr">
         <is>
-          <t>INATIVO- NIKSON DA SILVA ALVES</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2526" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2527">
       <c r="A2527" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2527" t="n">
-        <v>2819</v>
+        <v>2651</v>
       </c>
       <c r="C2527" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>INATIVO- NIKSON DA SILVA ALVES</t>
         </is>
       </c>
       <c r="D2527" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2528">
@@ -45927,87 +45927,87 @@
         </is>
       </c>
       <c r="B2528" t="n">
-        <v>2721</v>
+        <v>2819</v>
       </c>
       <c r="C2528" t="inlineStr">
         <is>
-          <t>H-TARCISIO ALVES DIAS</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2528" t="n">
-        <v>53</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2529">
       <c r="A2529" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2529" t="n">
-        <v>2746</v>
+        <v>2721</v>
       </c>
       <c r="C2529" t="inlineStr">
         <is>
-          <t>HERTZ CE - FCO DOUGLAS ALVES - INATIVO</t>
+          <t>H-TARCISIO ALVES DIAS</t>
         </is>
       </c>
       <c r="D2529" t="n">
-        <v>111</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2530">
       <c r="A2530" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2530" t="n">
-        <v>2699</v>
+        <v>2746</v>
       </c>
       <c r="C2530" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>HERTZ CE - FCO DOUGLAS ALVES - INATIVO</t>
         </is>
       </c>
       <c r="D2530" t="n">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2531">
       <c r="A2531" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2531" t="n">
-        <v>2700</v>
+        <v>2699</v>
       </c>
       <c r="C2531" t="inlineStr">
         <is>
-          <t>HERTZ CE - ROBSON LEITE - INATIVO</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2531" t="n">
-        <v>111</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2532">
       <c r="A2532" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2532" t="n">
-        <v>2706</v>
+        <v>2700</v>
       </c>
       <c r="C2532" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>HERTZ CE - ROBSON LEITE - INATIVO</t>
         </is>
       </c>
       <c r="D2532" t="n">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2533">
@@ -46017,11 +46017,11 @@
         </is>
       </c>
       <c r="B2533" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2533" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2533" t="n">
@@ -46031,127 +46031,127 @@
     <row r="2534">
       <c r="A2534" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2534" t="n">
-        <v>2693</v>
+        <v>2707</v>
       </c>
       <c r="C2534" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2534" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2535">
       <c r="A2535" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2535" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2535" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2535" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2536">
       <c r="A2536" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2536" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2536" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2536" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2537">
       <c r="A2537" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2537" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2537" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2537" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2538">
       <c r="A2538" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2538" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2538" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2538" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2539">
       <c r="A2539" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2539" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2539" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2539" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2540">
       <c r="A2540" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2540" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2540" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2540" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2541">
@@ -46161,11 +46161,11 @@
         </is>
       </c>
       <c r="B2541" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2541" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2541" t="n">
@@ -46175,37 +46175,37 @@
     <row r="2542">
       <c r="A2542" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2542" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2542" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2542" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2543">
       <c r="A2543" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2543" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2543" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2543" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2544">
@@ -46215,15 +46215,15 @@
         </is>
       </c>
       <c r="B2544" t="n">
-        <v>2774</v>
+        <v>2773</v>
       </c>
       <c r="C2544" t="inlineStr">
         <is>
-          <t>FRANCISCO MANOEL DE SOUSA (HERTZ)</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2544" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2545">
@@ -46233,15 +46233,15 @@
         </is>
       </c>
       <c r="B2545" t="n">
-        <v>2787</v>
+        <v>2774</v>
       </c>
       <c r="C2545" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>FRANCISCO MANOEL DE SOUSA (HERTZ)</t>
         </is>
       </c>
       <c r="D2545" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2546">
@@ -46251,33 +46251,33 @@
         </is>
       </c>
       <c r="B2546" t="n">
-        <v>2648</v>
+        <v>2787</v>
       </c>
       <c r="C2546" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2546" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2547">
       <c r="A2547" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2547" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2547" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2547" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2548">
@@ -46287,15 +46287,15 @@
         </is>
       </c>
       <c r="B2548" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2548" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2548" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2549">
@@ -46305,11 +46305,11 @@
         </is>
       </c>
       <c r="B2549" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2549" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2549" t="n">
@@ -46323,15 +46323,15 @@
         </is>
       </c>
       <c r="B2550" t="n">
-        <v>2784</v>
+        <v>2780</v>
       </c>
       <c r="C2550" t="inlineStr">
         <is>
-          <t>H-LORENA MARIA DA SILVA COSTA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2550" t="n">
-        <v>52</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2551">
@@ -46341,11 +46341,11 @@
         </is>
       </c>
       <c r="B2551" t="n">
-        <v>2785</v>
+        <v>2784</v>
       </c>
       <c r="C2551" t="inlineStr">
         <is>
-          <t>H-MARCOS VINICIUS GONCALVES MIRANDA</t>
+          <t>H-LORENA MARIA DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D2551" t="n">
@@ -46359,33 +46359,33 @@
         </is>
       </c>
       <c r="B2552" t="n">
-        <v>2786</v>
+        <v>2785</v>
       </c>
       <c r="C2552" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>H-MARCOS VINICIUS GONCALVES MIRANDA</t>
         </is>
       </c>
       <c r="D2552" t="n">
-        <v>100</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2553">
       <c r="A2553" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2553" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2553" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2553" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2554">
@@ -46395,15 +46395,15 @@
         </is>
       </c>
       <c r="B2554" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2554" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2554" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2555">
@@ -46413,11 +46413,11 @@
         </is>
       </c>
       <c r="B2555" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2555" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2555" t="n">
@@ -46427,73 +46427,73 @@
     <row r="2556">
       <c r="A2556" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2556" t="n">
-        <v>2763</v>
+        <v>2734</v>
       </c>
       <c r="C2556" t="inlineStr">
         <is>
-          <t>HERTZ CE- ANT GILSON FERREIRA DE ALENCAR</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2556" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2557">
       <c r="A2557" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2557" t="n">
-        <v>2764</v>
+        <v>2763</v>
       </c>
       <c r="C2557" t="inlineStr">
         <is>
-          <t>H-VAGO LUIZ CLAUDIO FREITAS SOBRAL</t>
+          <t>HERTZ CE- ANT GILSON FERREIRA DE ALENCAR</t>
         </is>
       </c>
       <c r="D2557" t="n">
-        <v>52</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2558">
       <c r="A2558" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2558" t="n">
-        <v>2782</v>
+        <v>2764</v>
       </c>
       <c r="C2558" t="inlineStr">
         <is>
-          <t>HERTZ CE - AMANDA DA SILVA BATISTA</t>
+          <t>H-VAGO LUIZ CLAUDIO FREITAS SOBRAL</t>
         </is>
       </c>
       <c r="D2558" t="n">
-        <v>111</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2559">
       <c r="A2559" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2559" t="n">
-        <v>2742</v>
+        <v>2782</v>
       </c>
       <c r="C2559" t="inlineStr">
         <is>
-          <t>MARCUS VINICIUS C. DE AZEVEDO - FARMA</t>
+          <t>HERTZ CE - AMANDA DA SILVA BATISTA</t>
         </is>
       </c>
       <c r="D2559" t="n">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2560">
@@ -46503,15 +46503,15 @@
         </is>
       </c>
       <c r="B2560" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2560" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>MARCUS VINICIUS C. DE AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2560" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2561">
@@ -46521,15 +46521,15 @@
         </is>
       </c>
       <c r="B2561" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2561" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2561" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2562">
@@ -46539,11 +46539,11 @@
         </is>
       </c>
       <c r="B2562" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2562" t="inlineStr">
         <is>
-          <t>BRENO ALLAN DE JESUS - FARM (SSA CENTRO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2562" t="n">
@@ -46557,11 +46557,11 @@
         </is>
       </c>
       <c r="B2563" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2563" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>BRENO ALLAN DE JESUS - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2563" t="n">
@@ -46575,11 +46575,11 @@
         </is>
       </c>
       <c r="B2564" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2564" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2564" t="n">
@@ -46589,73 +46589,73 @@
     <row r="2565">
       <c r="A2565" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2565" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2565" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2565" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2566">
       <c r="A2566" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2566" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2566" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2566" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2567">
       <c r="A2567" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2567" t="n">
-        <v>2702</v>
+        <v>2690</v>
       </c>
       <c r="C2567" t="inlineStr">
         <is>
-          <t>H-RICARDO MACAUBAS BOAVENTURA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2567" t="n">
-        <v>53</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2568">
       <c r="A2568" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2568" t="n">
-        <v>2696</v>
+        <v>2702</v>
       </c>
       <c r="C2568" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>H-RICARDO MACAUBAS BOAVENTURA</t>
         </is>
       </c>
       <c r="D2568" t="n">
-        <v>69</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2569">
@@ -46665,11 +46665,11 @@
         </is>
       </c>
       <c r="B2569" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2569" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2569" t="n">
@@ -46683,11 +46683,11 @@
         </is>
       </c>
       <c r="B2570" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2570" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2570" t="n">
@@ -46697,19 +46697,19 @@
     <row r="2571">
       <c r="A2571" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2571" t="n">
-        <v>2770</v>
+        <v>2698</v>
       </c>
       <c r="C2571" t="inlineStr">
         <is>
-          <t>HERTZ CE - LUANDA MARCELINO DE OLIVEIRA</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2571" t="n">
-        <v>111</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2572">
@@ -46719,11 +46719,11 @@
         </is>
       </c>
       <c r="B2572" t="n">
-        <v>2771</v>
+        <v>2770</v>
       </c>
       <c r="C2572" t="inlineStr">
         <is>
-          <t>HERTZ CE - EDUARDO BEZERRA DE SOUSA</t>
+          <t>HERTZ CE - LUANDA MARCELINO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2572" t="n">
@@ -46733,19 +46733,19 @@
     <row r="2573">
       <c r="A2573" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2573" t="n">
-        <v>2775</v>
+        <v>2771</v>
       </c>
       <c r="C2573" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>HERTZ CE - EDUARDO BEZERRA DE SOUSA</t>
         </is>
       </c>
       <c r="D2573" t="n">
-        <v>38</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2574">
@@ -46755,11 +46755,11 @@
         </is>
       </c>
       <c r="B2574" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2574" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2574" t="n">
@@ -46773,11 +46773,11 @@
         </is>
       </c>
       <c r="B2575" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2575" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2575" t="n">
@@ -46791,11 +46791,11 @@
         </is>
       </c>
       <c r="B2576" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2576" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2576" t="n">
@@ -46809,15 +46809,15 @@
         </is>
       </c>
       <c r="B2577" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2577" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2577" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2578">
@@ -46827,15 +46827,15 @@
         </is>
       </c>
       <c r="B2578" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2578" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2578" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2579">
@@ -46845,11 +46845,11 @@
         </is>
       </c>
       <c r="B2579" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2579" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2579" t="n">
@@ -46859,37 +46859,37 @@
     <row r="2580">
       <c r="A2580" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2580" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2580" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2580" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2581">
       <c r="A2581" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2581" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2581" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2581" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2582">
@@ -46899,50 +46899,68 @@
         </is>
       </c>
       <c r="B2582" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2582" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2582" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2583">
       <c r="A2583" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2583" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2583" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2583" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2584">
       <c r="A2584" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2584" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2584" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2584" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2585">
+      <c r="A2585" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B2584" t="n">
+      <c r="B2585" t="n">
         <v>2801</v>
       </c>
-      <c r="C2584" t="inlineStr">
+      <c r="C2585" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2584" t="n">
+      <c r="D2585" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 15:57:58
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2585"/>
+  <dimension ref="A1:D2587"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44195,19 +44195,19 @@
     <row r="2432">
       <c r="A2432" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2747</v>
+        <v>2824</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2432" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2433">
@@ -44217,11 +44217,11 @@
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>WILSON PORTUGAL AZEVEDO FILHO - FARMA</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2433" t="n">
@@ -44231,73 +44231,73 @@
     <row r="2434">
       <c r="A2434" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2766</v>
+        <v>2748</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>WILSON PORTUGAL AZEVEDO FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2434" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2435">
       <c r="A2435" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2767</v>
+        <v>2766</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2435" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2436">
       <c r="A2436" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2688</v>
+        <v>2767</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2436" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2437">
       <c r="A2437" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2694</v>
+        <v>2688</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2437" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2438">
@@ -44307,15 +44307,15 @@
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2714</v>
+        <v>2694</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2438" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2439">
@@ -44325,15 +44325,15 @@
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2722</v>
+        <v>2714</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2439" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2440">
@@ -44343,15 +44343,15 @@
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2440" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2441">
@@ -44361,15 +44361,15 @@
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2803</v>
+        <v>2723</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2441" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2442">
@@ -44379,11 +44379,11 @@
         </is>
       </c>
       <c r="B2442" t="n">
-        <v>2804</v>
+        <v>2803</v>
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2442" t="n">
@@ -44397,15 +44397,15 @@
         </is>
       </c>
       <c r="B2443" t="n">
-        <v>2809</v>
+        <v>2804</v>
       </c>
       <c r="C2443" t="inlineStr">
         <is>
-          <t>H-LUCILENE SANTOS DE MELO DAMASCENA</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2443" t="n">
-        <v>115</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2444">
@@ -44415,69 +44415,69 @@
         </is>
       </c>
       <c r="B2444" t="n">
-        <v>2811</v>
+        <v>2809</v>
       </c>
       <c r="C2444" t="inlineStr">
         <is>
-          <t>H-ROSEANE SILVA FERREIRA</t>
+          <t>H-LUCILENE SANTOS DE MELO DAMASCENA</t>
         </is>
       </c>
       <c r="D2444" t="n">
-        <v>52</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2445">
       <c r="A2445" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2445" t="n">
-        <v>2647</v>
+        <v>2811</v>
       </c>
       <c r="C2445" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>H-ROSEANE SILVA FERREIRA</t>
         </is>
       </c>
       <c r="D2445" t="n">
-        <v>147</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2446">
       <c r="A2446" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2446" t="n">
-        <v>2661</v>
+        <v>2647</v>
       </c>
       <c r="C2446" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2446" t="n">
-        <v>76</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2447">
       <c r="A2447" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2447" t="n">
-        <v>2686</v>
+        <v>2661</v>
       </c>
       <c r="C2447" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2447" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2448">
@@ -44487,11 +44487,11 @@
         </is>
       </c>
       <c r="B2448" t="n">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="C2448" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2448" t="n">
@@ -44501,91 +44501,91 @@
     <row r="2449">
       <c r="A2449" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2449" t="n">
-        <v>2681</v>
+        <v>2687</v>
       </c>
       <c r="C2449" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2449" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2450">
       <c r="A2450" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2450" t="n">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="C2450" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2450" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2451">
       <c r="A2451" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2451" t="n">
-        <v>2677</v>
+        <v>2682</v>
       </c>
       <c r="C2451" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2451" t="n">
-        <v>72</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2452">
       <c r="A2452" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2452" t="n">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="C2452" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2452" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2453">
       <c r="A2453" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2453" t="n">
-        <v>2735</v>
+        <v>2678</v>
       </c>
       <c r="C2453" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2453" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2454">
@@ -44595,15 +44595,15 @@
         </is>
       </c>
       <c r="B2454" t="n">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="C2454" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2454" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2455">
@@ -44613,15 +44613,15 @@
         </is>
       </c>
       <c r="B2455" t="n">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C2455" t="inlineStr">
         <is>
-          <t>MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2455" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2456">
@@ -44631,15 +44631,15 @@
         </is>
       </c>
       <c r="B2456" t="n">
-        <v>2743</v>
+        <v>2737</v>
       </c>
       <c r="C2456" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2456" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2457">
@@ -44649,11 +44649,11 @@
         </is>
       </c>
       <c r="B2457" t="n">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="C2457" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2457" t="n">
@@ -44667,15 +44667,15 @@
         </is>
       </c>
       <c r="B2458" t="n">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="C2458" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2458" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2459">
@@ -44685,15 +44685,15 @@
         </is>
       </c>
       <c r="B2459" t="n">
-        <v>2761</v>
+        <v>2745</v>
       </c>
       <c r="C2459" t="inlineStr">
         <is>
-          <t>H-SANON MOREIRA SOUZA</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2459" t="n">
-        <v>53</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2460">
@@ -44703,11 +44703,11 @@
         </is>
       </c>
       <c r="B2460" t="n">
-        <v>2762</v>
+        <v>2761</v>
       </c>
       <c r="C2460" t="inlineStr">
         <is>
-          <t>H-GILSON PINTO ALVES</t>
+          <t>H-SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D2460" t="n">
@@ -44721,51 +44721,51 @@
         </is>
       </c>
       <c r="B2461" t="n">
-        <v>2783</v>
+        <v>2762</v>
       </c>
       <c r="C2461" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>H-GILSON PINTO ALVES</t>
         </is>
       </c>
       <c r="D2461" t="n">
-        <v>95</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2462">
       <c r="A2462" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2462" t="n">
-        <v>2768</v>
+        <v>2783</v>
       </c>
       <c r="C2462" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2462" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2463">
       <c r="A2463" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2463" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2463" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2463" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2464">
@@ -44775,33 +44775,33 @@
         </is>
       </c>
       <c r="B2464" t="n">
-        <v>2750</v>
+        <v>2703</v>
       </c>
       <c r="C2464" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2464" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2465">
       <c r="A2465" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2465" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2465" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2465" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2466">
@@ -44811,51 +44811,51 @@
         </is>
       </c>
       <c r="B2466" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2466" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2466" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2467">
       <c r="A2467" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2467" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2467" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2467" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2468">
       <c r="A2468" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2468" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2468" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2468" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2469">
@@ -44865,15 +44865,15 @@
         </is>
       </c>
       <c r="B2469" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2469" t="inlineStr">
         <is>
-          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2469" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2470">
@@ -44883,11 +44883,11 @@
         </is>
       </c>
       <c r="B2470" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2470" t="inlineStr">
         <is>
-          <t>DANIELY PEREIRA PINHEIRO</t>
+          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
         </is>
       </c>
       <c r="D2470" t="n">
@@ -44897,19 +44897,19 @@
     <row r="2471">
       <c r="A2471" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2471" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2471" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY PEREIRA PINHEIRO</t>
         </is>
       </c>
       <c r="D2471" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2472">
@@ -44919,11 +44919,11 @@
         </is>
       </c>
       <c r="B2472" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2472" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2472" t="n">
@@ -44937,11 +44937,11 @@
         </is>
       </c>
       <c r="B2473" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2473" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2473" t="n">
@@ -44955,11 +44955,11 @@
         </is>
       </c>
       <c r="B2474" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2474" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2474" t="n">
@@ -44969,91 +44969,91 @@
     <row r="2475">
       <c r="A2475" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B2475" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2475" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2475" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2476">
       <c r="A2476" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2476" t="n">
-        <v>2765</v>
+        <v>2820</v>
       </c>
       <c r="C2476" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2476" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2477">
       <c r="A2477" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2477" t="n">
-        <v>2741</v>
+        <v>2765</v>
       </c>
       <c r="C2477" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2477" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2478">
       <c r="A2478" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2478" t="n">
-        <v>2695</v>
+        <v>2741</v>
       </c>
       <c r="C2478" t="inlineStr">
         <is>
-          <t>HERTZ CE - RODRIGO ALVES DE MESQUITA</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2478" t="n">
-        <v>111</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2479">
       <c r="A2479" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2479" t="n">
-        <v>2758</v>
+        <v>2695</v>
       </c>
       <c r="C2479" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>HERTZ CE - RODRIGO ALVES DE MESQUITA</t>
         </is>
       </c>
       <c r="D2479" t="n">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2480">
@@ -45063,51 +45063,51 @@
         </is>
       </c>
       <c r="B2480" t="n">
-        <v>2659</v>
+        <v>2758</v>
       </c>
       <c r="C2480" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2480" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2481">
       <c r="A2481" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2481" t="n">
-        <v>2669</v>
+        <v>2659</v>
       </c>
       <c r="C2481" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2481" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2482">
       <c r="A2482" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2482" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2482" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2482" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2483">
@@ -45117,33 +45117,33 @@
         </is>
       </c>
       <c r="B2483" t="n">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="C2483" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO VIRIATO SANTOS - FARMA</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2483" t="n">
-        <v>50</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2484">
       <c r="A2484" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2484" t="n">
-        <v>2676</v>
+        <v>2673</v>
       </c>
       <c r="C2484" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO  CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2484" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2485">
@@ -45153,87 +45153,87 @@
         </is>
       </c>
       <c r="B2485" t="n">
-        <v>2760</v>
+        <v>2676</v>
       </c>
       <c r="C2485" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2485" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2486">
       <c r="A2486" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2486" t="n">
-        <v>2818</v>
+        <v>2760</v>
       </c>
       <c r="C2486" t="inlineStr">
         <is>
-          <t>HERTZ CE -  FRANCISCO RILDES T OLIVEIRA</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2486" t="n">
-        <v>111</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2487">
       <c r="A2487" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2487" t="n">
-        <v>2823</v>
+        <v>2818</v>
       </c>
       <c r="C2487" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>HERTZ CE -  FRANCISCO RILDES T OLIVEIRA</t>
         </is>
       </c>
       <c r="D2487" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2488">
       <c r="A2488" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2488" t="n">
-        <v>2792</v>
+        <v>2823</v>
       </c>
       <c r="C2488" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2488" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2489">
       <c r="A2489" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2489" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2489" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2489" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2490">
@@ -45243,15 +45243,15 @@
         </is>
       </c>
       <c r="B2490" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2490" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2490" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2491">
@@ -45261,15 +45261,15 @@
         </is>
       </c>
       <c r="B2491" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2491" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2491" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2492">
@@ -45279,15 +45279,15 @@
         </is>
       </c>
       <c r="B2492" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2492" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2492" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2493">
@@ -45297,11 +45297,11 @@
         </is>
       </c>
       <c r="B2493" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2493" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D2493" t="n">
@@ -45311,37 +45311,37 @@
     <row r="2494">
       <c r="A2494" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2494" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2494" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2494" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2495">
       <c r="A2495" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2495" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2495" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2495" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2496">
@@ -45351,11 +45351,11 @@
         </is>
       </c>
       <c r="B2496" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2496" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2496" t="n">
@@ -45365,55 +45365,55 @@
     <row r="2497">
       <c r="A2497" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2497" t="n">
-        <v>2642</v>
+        <v>2769</v>
       </c>
       <c r="C2497" t="inlineStr">
         <is>
-          <t>H-VAGO DESIREE BARROS DE CARVALHO</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2497" t="n">
-        <v>52</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2498">
       <c r="A2498" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2498" t="n">
-        <v>2649</v>
+        <v>2642</v>
       </c>
       <c r="C2498" t="inlineStr">
         <is>
-          <t>HERTZ PE - (VAGO/DIEGO CALABRIA)</t>
+          <t>H-VAGO DESIREE BARROS DE CARVALHO</t>
         </is>
       </c>
       <c r="D2498" t="n">
-        <v>142</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2499">
       <c r="A2499" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2499" t="n">
-        <v>2679</v>
+        <v>2649</v>
       </c>
       <c r="C2499" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>HERTZ PE - (VAGO/DIEGO CALABRIA)</t>
         </is>
       </c>
       <c r="D2499" t="n">
-        <v>69</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2500">
@@ -45423,11 +45423,11 @@
         </is>
       </c>
       <c r="B2500" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2500" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2500" t="n">
@@ -45437,19 +45437,19 @@
     <row r="2501">
       <c r="A2501" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2501" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2501" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2501" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2502">
@@ -45459,15 +45459,15 @@
         </is>
       </c>
       <c r="B2502" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2502" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2502" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2503">
@@ -45477,11 +45477,11 @@
         </is>
       </c>
       <c r="B2503" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2503" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2503" t="n">
@@ -45491,37 +45491,37 @@
     <row r="2504">
       <c r="A2504" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2504" t="n">
-        <v>2701</v>
+        <v>2817</v>
       </c>
       <c r="C2504" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2504" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2505">
       <c r="A2505" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2505" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2505" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2505" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2506">
@@ -45531,11 +45531,11 @@
         </is>
       </c>
       <c r="B2506" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2506" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2506" t="n">
@@ -45545,19 +45545,19 @@
     <row r="2507">
       <c r="A2507" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B2507" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2507" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2507" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2508">
@@ -45567,51 +45567,51 @@
         </is>
       </c>
       <c r="B2508" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2508" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2508" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2509">
       <c r="A2509" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2509" t="n">
-        <v>2788</v>
+        <v>2755</v>
       </c>
       <c r="C2509" t="inlineStr">
         <is>
-          <t>H-ARTHUR GV HERTZ</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2509" t="n">
-        <v>52</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2510">
       <c r="A2510" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2510" t="n">
-        <v>2665</v>
+        <v>2788</v>
       </c>
       <c r="C2510" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>H-ARTHUR GV HERTZ</t>
         </is>
       </c>
       <c r="D2510" t="n">
-        <v>141</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2511">
@@ -45621,15 +45621,15 @@
         </is>
       </c>
       <c r="B2511" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2511" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2511" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2512">
@@ -45639,15 +45639,15 @@
         </is>
       </c>
       <c r="B2512" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2512" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
         </is>
       </c>
       <c r="D2512" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2513">
@@ -45657,11 +45657,11 @@
         </is>
       </c>
       <c r="B2513" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2513" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2513" t="n">
@@ -45671,37 +45671,37 @@
     <row r="2514">
       <c r="A2514" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2514" t="n">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="C2514" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2514" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2515">
       <c r="A2515" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2515" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2515" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2515" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2516">
@@ -45711,11 +45711,11 @@
         </is>
       </c>
       <c r="B2516" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2516" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2516" t="n">
@@ -45729,15 +45729,15 @@
         </is>
       </c>
       <c r="B2517" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2517" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2517" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2518">
@@ -45747,11 +45747,11 @@
         </is>
       </c>
       <c r="B2518" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2518" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - HB</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2518" t="n">
@@ -45765,15 +45765,15 @@
         </is>
       </c>
       <c r="B2519" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2519" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - HB</t>
         </is>
       </c>
       <c r="D2519" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2520">
@@ -45783,51 +45783,51 @@
         </is>
       </c>
       <c r="B2520" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2520" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2520" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2521">
       <c r="A2521" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2521" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2521" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2521" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2522">
       <c r="A2522" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2522" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2522" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2522" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2523">
@@ -45837,33 +45837,33 @@
         </is>
       </c>
       <c r="B2523" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2523" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2523" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2524">
       <c r="A2524" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2524" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2524" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2524" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2525">
@@ -45873,69 +45873,69 @@
         </is>
       </c>
       <c r="B2525" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2525" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2525" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2526">
       <c r="A2526" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2526" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2526" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2526" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2527">
       <c r="A2527" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2527" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2527" t="inlineStr">
         <is>
-          <t>INATIVO- NIKSON DA SILVA ALVES</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2527" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2528">
       <c r="A2528" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2528" t="n">
-        <v>2819</v>
+        <v>2651</v>
       </c>
       <c r="C2528" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2528" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2529">
@@ -45945,87 +45945,87 @@
         </is>
       </c>
       <c r="B2529" t="n">
-        <v>2721</v>
+        <v>2819</v>
       </c>
       <c r="C2529" t="inlineStr">
         <is>
-          <t>H-TARCISIO ALVES DIAS</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2529" t="n">
-        <v>53</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2530">
       <c r="A2530" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2530" t="n">
-        <v>2746</v>
+        <v>2721</v>
       </c>
       <c r="C2530" t="inlineStr">
         <is>
-          <t>HERTZ CE - FCO DOUGLAS ALVES - INATIVO</t>
+          <t>H-TARCISIO ALVES DIAS</t>
         </is>
       </c>
       <c r="D2530" t="n">
-        <v>111</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2531">
       <c r="A2531" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2531" t="n">
-        <v>2699</v>
+        <v>2746</v>
       </c>
       <c r="C2531" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>HERTZ CE - FCO DOUGLAS ALVES - INATIVO</t>
         </is>
       </c>
       <c r="D2531" t="n">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2532">
       <c r="A2532" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2532" t="n">
-        <v>2700</v>
+        <v>2699</v>
       </c>
       <c r="C2532" t="inlineStr">
         <is>
-          <t>HERTZ CE - ROBSON LEITE - INATIVO</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2532" t="n">
-        <v>111</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2533">
       <c r="A2533" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2533" t="n">
-        <v>2706</v>
+        <v>2700</v>
       </c>
       <c r="C2533" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>HERTZ CE - ROBSON LEITE - INATIVO</t>
         </is>
       </c>
       <c r="D2533" t="n">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2534">
@@ -46035,11 +46035,11 @@
         </is>
       </c>
       <c r="B2534" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2534" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2534" t="n">
@@ -46049,127 +46049,127 @@
     <row r="2535">
       <c r="A2535" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2535" t="n">
-        <v>2693</v>
+        <v>2707</v>
       </c>
       <c r="C2535" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2535" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2536">
       <c r="A2536" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2536" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2536" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2536" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2537">
       <c r="A2537" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2537" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2537" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2537" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2538">
       <c r="A2538" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2538" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2538" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2538" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2539">
       <c r="A2539" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2539" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2539" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2539" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2540">
       <c r="A2540" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2540" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2540" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2540" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2541">
       <c r="A2541" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2541" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2541" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2541" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2542">
@@ -46179,11 +46179,11 @@
         </is>
       </c>
       <c r="B2542" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2542" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2542" t="n">
@@ -46193,37 +46193,37 @@
     <row r="2543">
       <c r="A2543" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2543" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2543" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2543" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2544">
       <c r="A2544" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2544" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2544" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2544" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2545">
@@ -46233,15 +46233,15 @@
         </is>
       </c>
       <c r="B2545" t="n">
-        <v>2774</v>
+        <v>2773</v>
       </c>
       <c r="C2545" t="inlineStr">
         <is>
-          <t>FRANCISCO MANOEL DE SOUSA (HERTZ)</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2545" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2546">
@@ -46251,15 +46251,15 @@
         </is>
       </c>
       <c r="B2546" t="n">
-        <v>2787</v>
+        <v>2774</v>
       </c>
       <c r="C2546" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>FRANCISCO MANOEL DE SOUSA (HERTZ)</t>
         </is>
       </c>
       <c r="D2546" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2547">
@@ -46269,51 +46269,51 @@
         </is>
       </c>
       <c r="B2547" t="n">
-        <v>2648</v>
+        <v>2825</v>
       </c>
       <c r="C2547" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2547" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2548">
       <c r="A2548" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2548" t="n">
-        <v>2666</v>
+        <v>2787</v>
       </c>
       <c r="C2548" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2548" t="n">
-        <v>63</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2549">
       <c r="A2549" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2549" t="n">
-        <v>2779</v>
+        <v>2648</v>
       </c>
       <c r="C2549" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2549" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2550">
@@ -46323,15 +46323,15 @@
         </is>
       </c>
       <c r="B2550" t="n">
-        <v>2780</v>
+        <v>2666</v>
       </c>
       <c r="C2550" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2550" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2551">
@@ -46341,15 +46341,15 @@
         </is>
       </c>
       <c r="B2551" t="n">
-        <v>2784</v>
+        <v>2779</v>
       </c>
       <c r="C2551" t="inlineStr">
         <is>
-          <t>H-LORENA MARIA DA SILVA COSTA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2551" t="n">
-        <v>52</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2552">
@@ -46359,15 +46359,15 @@
         </is>
       </c>
       <c r="B2552" t="n">
-        <v>2785</v>
+        <v>2780</v>
       </c>
       <c r="C2552" t="inlineStr">
         <is>
-          <t>H-MARCOS VINICIUS GONCALVES MIRANDA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2552" t="n">
-        <v>52</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2553">
@@ -46377,51 +46377,51 @@
         </is>
       </c>
       <c r="B2553" t="n">
-        <v>2786</v>
+        <v>2784</v>
       </c>
       <c r="C2553" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>H-LORENA MARIA DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D2553" t="n">
-        <v>100</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2554">
       <c r="A2554" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2554" t="n">
-        <v>2660</v>
+        <v>2785</v>
       </c>
       <c r="C2554" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>H-MARCOS VINICIUS GONCALVES MIRANDA</t>
         </is>
       </c>
       <c r="D2554" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2555">
       <c r="A2555" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2555" t="n">
-        <v>2716</v>
+        <v>2786</v>
       </c>
       <c r="C2555" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2555" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2556">
@@ -46431,51 +46431,51 @@
         </is>
       </c>
       <c r="B2556" t="n">
-        <v>2734</v>
+        <v>2660</v>
       </c>
       <c r="C2556" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2556" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2557">
       <c r="A2557" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2557" t="n">
-        <v>2763</v>
+        <v>2716</v>
       </c>
       <c r="C2557" t="inlineStr">
         <is>
-          <t>HERTZ CE- ANT GILSON FERREIRA DE ALENCAR</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2557" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2558">
       <c r="A2558" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2558" t="n">
-        <v>2764</v>
+        <v>2734</v>
       </c>
       <c r="C2558" t="inlineStr">
         <is>
-          <t>H-VAGO LUIZ CLAUDIO FREITAS SOBRAL</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2558" t="n">
-        <v>52</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2559">
@@ -46485,11 +46485,11 @@
         </is>
       </c>
       <c r="B2559" t="n">
-        <v>2782</v>
+        <v>2763</v>
       </c>
       <c r="C2559" t="inlineStr">
         <is>
-          <t>HERTZ CE - AMANDA DA SILVA BATISTA</t>
+          <t>HERTZ CE- ANT GILSON FERREIRA DE ALENCAR</t>
         </is>
       </c>
       <c r="D2559" t="n">
@@ -46503,33 +46503,33 @@
         </is>
       </c>
       <c r="B2560" t="n">
-        <v>2742</v>
+        <v>2764</v>
       </c>
       <c r="C2560" t="inlineStr">
         <is>
-          <t>MARCUS VINICIUS C. DE AZEVEDO - FARMA</t>
+          <t>H-VAGO LUIZ CLAUDIO FREITAS SOBRAL</t>
         </is>
       </c>
       <c r="D2560" t="n">
-        <v>95</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2561">
       <c r="A2561" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2561" t="n">
-        <v>2794</v>
+        <v>2782</v>
       </c>
       <c r="C2561" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>HERTZ CE - AMANDA DA SILVA BATISTA</t>
         </is>
       </c>
       <c r="D2561" t="n">
-        <v>98</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2562">
@@ -46539,11 +46539,11 @@
         </is>
       </c>
       <c r="B2562" t="n">
-        <v>2795</v>
+        <v>2742</v>
       </c>
       <c r="C2562" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2562" t="n">
@@ -46557,15 +46557,15 @@
         </is>
       </c>
       <c r="B2563" t="n">
-        <v>2796</v>
+        <v>2794</v>
       </c>
       <c r="C2563" t="inlineStr">
         <is>
-          <t>BRENO ALLAN DE JESUS - FARM (SSA CENTRO)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2563" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2564">
@@ -46575,11 +46575,11 @@
         </is>
       </c>
       <c r="B2564" t="n">
-        <v>2797</v>
+        <v>2795</v>
       </c>
       <c r="C2564" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2564" t="n">
@@ -46593,11 +46593,11 @@
         </is>
       </c>
       <c r="B2565" t="n">
-        <v>2798</v>
+        <v>2796</v>
       </c>
       <c r="C2565" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>BRENO ALLAN DE JESUS - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2565" t="n">
@@ -46607,91 +46607,91 @@
     <row r="2566">
       <c r="A2566" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2566" t="n">
-        <v>2668</v>
+        <v>2797</v>
       </c>
       <c r="C2566" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2566" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2567">
       <c r="A2567" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2567" t="n">
-        <v>2690</v>
+        <v>2798</v>
       </c>
       <c r="C2567" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2567" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2568">
       <c r="A2568" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2568" t="n">
-        <v>2702</v>
+        <v>2668</v>
       </c>
       <c r="C2568" t="inlineStr">
         <is>
-          <t>H-RICARDO MACAUBAS BOAVENTURA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2568" t="n">
-        <v>53</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2569">
       <c r="A2569" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2569" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2569" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2569" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2570">
       <c r="A2570" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2570" t="n">
-        <v>2697</v>
+        <v>2702</v>
       </c>
       <c r="C2570" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>H-RICARDO MACAUBAS BOAVENTURA</t>
         </is>
       </c>
       <c r="D2570" t="n">
-        <v>69</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2571">
@@ -46701,11 +46701,11 @@
         </is>
       </c>
       <c r="B2571" t="n">
-        <v>2698</v>
+        <v>2696</v>
       </c>
       <c r="C2571" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2571" t="n">
@@ -46715,73 +46715,73 @@
     <row r="2572">
       <c r="A2572" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2572" t="n">
-        <v>2770</v>
+        <v>2697</v>
       </c>
       <c r="C2572" t="inlineStr">
         <is>
-          <t>HERTZ CE - LUANDA MARCELINO DE OLIVEIRA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2572" t="n">
-        <v>111</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2573">
       <c r="A2573" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2573" t="n">
-        <v>2771</v>
+        <v>2698</v>
       </c>
       <c r="C2573" t="inlineStr">
         <is>
-          <t>HERTZ CE - EDUARDO BEZERRA DE SOUSA</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2573" t="n">
-        <v>111</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2574">
       <c r="A2574" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2574" t="n">
-        <v>2775</v>
+        <v>2770</v>
       </c>
       <c r="C2574" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>HERTZ CE - LUANDA MARCELINO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2574" t="n">
-        <v>38</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2575">
       <c r="A2575" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2575" t="n">
-        <v>2776</v>
+        <v>2771</v>
       </c>
       <c r="C2575" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>HERTZ CE - EDUARDO BEZERRA DE SOUSA</t>
         </is>
       </c>
       <c r="D2575" t="n">
-        <v>38</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2576">
@@ -46791,11 +46791,11 @@
         </is>
       </c>
       <c r="B2576" t="n">
-        <v>2777</v>
+        <v>2775</v>
       </c>
       <c r="C2576" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2576" t="n">
@@ -46809,11 +46809,11 @@
         </is>
       </c>
       <c r="B2577" t="n">
-        <v>2778</v>
+        <v>2776</v>
       </c>
       <c r="C2577" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2577" t="n">
@@ -46827,15 +46827,15 @@
         </is>
       </c>
       <c r="B2578" t="n">
-        <v>2781</v>
+        <v>2777</v>
       </c>
       <c r="C2578" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2578" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2579">
@@ -46845,11 +46845,11 @@
         </is>
       </c>
       <c r="B2579" t="n">
-        <v>2822</v>
+        <v>2778</v>
       </c>
       <c r="C2579" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2579" t="n">
@@ -46863,33 +46863,33 @@
         </is>
       </c>
       <c r="B2580" t="n">
-        <v>2740</v>
+        <v>2781</v>
       </c>
       <c r="C2580" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2580" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2581">
       <c r="A2581" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2581" t="n">
-        <v>2710</v>
+        <v>2822</v>
       </c>
       <c r="C2581" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2581" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2582">
@@ -46899,51 +46899,51 @@
         </is>
       </c>
       <c r="B2582" t="n">
-        <v>2711</v>
+        <v>2740</v>
       </c>
       <c r="C2582" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2582" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2583">
       <c r="A2583" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2583" t="n">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="C2583" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2583" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2584">
       <c r="A2584" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2584" t="n">
-        <v>2717</v>
+        <v>2711</v>
       </c>
       <c r="C2584" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2584" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2585">
@@ -46953,14 +46953,50 @@
         </is>
       </c>
       <c r="B2585" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2585" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2585" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2586">
+      <c r="A2586" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2586" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2586" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2586" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2587">
+      <c r="A2587" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2587" t="n">
         <v>2801</v>
       </c>
-      <c r="C2585" t="inlineStr">
+      <c r="C2587" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2585" t="n">
+      <c r="D2587" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:00:06
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2422"/>
+  <dimension ref="A1:D2423"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41513,37 +41513,37 @@
     <row r="2283">
       <c r="A2283" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2283" t="n">
-        <v>2756</v>
+        <v>2827</v>
       </c>
       <c r="C2283" t="inlineStr">
         <is>
-          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
+          <t>JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2283" t="n">
-        <v>39</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2284">
       <c r="A2284" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2284" t="n">
-        <v>2813</v>
+        <v>2756</v>
       </c>
       <c r="C2284" t="inlineStr">
         <is>
-          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
+          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
         </is>
       </c>
       <c r="D2284" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2285">
@@ -41553,15 +41553,15 @@
         </is>
       </c>
       <c r="B2285" t="n">
-        <v>2738</v>
+        <v>2813</v>
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
+          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="D2285" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2286">
@@ -41571,11 +41571,11 @@
         </is>
       </c>
       <c r="B2286" t="n">
-        <v>2739</v>
+        <v>2738</v>
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
+          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2286" t="n">
@@ -41589,33 +41589,33 @@
         </is>
       </c>
       <c r="B2287" t="n">
-        <v>2824</v>
+        <v>2739</v>
       </c>
       <c r="C2287" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2287" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2288">
       <c r="A2288" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2288" t="n">
-        <v>2747</v>
+        <v>2824</v>
       </c>
       <c r="C2288" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2288" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2289">
@@ -41625,11 +41625,11 @@
         </is>
       </c>
       <c r="B2289" t="n">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="C2289" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2289" t="n">
@@ -41639,73 +41639,73 @@
     <row r="2290">
       <c r="A2290" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2290" t="n">
-        <v>2766</v>
+        <v>2748</v>
       </c>
       <c r="C2290" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2290" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2291">
       <c r="A2291" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2291" t="n">
-        <v>2767</v>
+        <v>2766</v>
       </c>
       <c r="C2291" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2291" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2292">
       <c r="A2292" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2688</v>
+        <v>2767</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2292" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2293">
       <c r="A2293" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2694</v>
+        <v>2688</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2293" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2294">
@@ -41715,15 +41715,15 @@
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2714</v>
+        <v>2694</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2294" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2295">
@@ -41733,15 +41733,15 @@
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2722</v>
+        <v>2714</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2295" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2296">
@@ -41751,15 +41751,15 @@
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2296" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2297">
@@ -41769,15 +41769,15 @@
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2803</v>
+        <v>2723</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2298">
@@ -41787,11 +41787,11 @@
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2804</v>
+        <v>2803</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2298" t="n">
@@ -41801,55 +41801,55 @@
     <row r="2299">
       <c r="A2299" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2647</v>
+        <v>2804</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2299" t="n">
-        <v>147</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2300">
       <c r="A2300" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2661</v>
+        <v>2647</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>76</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2301">
       <c r="A2301" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2686</v>
+        <v>2661</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2302">
@@ -41859,11 +41859,11 @@
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2302" t="n">
@@ -41873,109 +41873,109 @@
     <row r="2303">
       <c r="A2303" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2681</v>
+        <v>2687</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2303" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2304">
       <c r="A2304" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2304" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2826</v>
+        <v>2682</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2305" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2677</v>
+        <v>2826</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2735</v>
+        <v>2678</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2309">
@@ -41985,15 +41985,15 @@
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2309" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2310">
@@ -42003,15 +42003,15 @@
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2311">
@@ -42021,15 +42021,15 @@
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2743</v>
+        <v>2737</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2312">
@@ -42039,11 +42039,11 @@
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2312" t="n">
@@ -42057,15 +42057,15 @@
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2314">
@@ -42075,51 +42075,51 @@
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2783</v>
+        <v>2745</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2315">
       <c r="A2315" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2768</v>
+        <v>2783</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2316">
       <c r="A2316" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2317">
@@ -42129,33 +42129,33 @@
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2750</v>
+        <v>2703</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2318">
       <c r="A2318" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2319">
@@ -42165,51 +42165,51 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2320">
       <c r="A2320" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2321">
       <c r="A2321" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2322">
@@ -42219,15 +42219,15 @@
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2323">
@@ -42237,11 +42237,11 @@
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>DANIELY PEREIRA PINHEIRO</t>
+          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
         </is>
       </c>
       <c r="D2323" t="n">
@@ -42251,19 +42251,19 @@
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY PEREIRA PINHEIRO</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2325">
@@ -42273,11 +42273,11 @@
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2325" t="n">
@@ -42291,11 +42291,11 @@
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2326" t="n">
@@ -42309,11 +42309,11 @@
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2327" t="n">
@@ -42323,73 +42323,73 @@
     <row r="2328">
       <c r="A2328" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2765</v>
+        <v>2820</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2741</v>
+        <v>2765</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2758</v>
+        <v>2741</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2332">
@@ -42399,51 +42399,51 @@
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2659</v>
+        <v>2758</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2332" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2333">
       <c r="A2333" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2669</v>
+        <v>2659</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2333" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2334">
       <c r="A2334" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2334" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2335">
@@ -42453,33 +42453,33 @@
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>VAGO  CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2335" t="n">
-        <v>50</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2336">
       <c r="A2336" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2676</v>
+        <v>2673</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2336" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2337">
@@ -42489,69 +42489,69 @@
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2760</v>
+        <v>2676</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2338">
       <c r="A2338" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2823</v>
+        <v>2760</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>80</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2792</v>
+        <v>2823</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2341">
@@ -42561,15 +42561,15 @@
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2342">
@@ -42579,15 +42579,15 @@
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2343">
@@ -42597,15 +42597,15 @@
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2344">
@@ -42615,11 +42615,11 @@
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D2344" t="n">
@@ -42629,37 +42629,37 @@
     <row r="2345">
       <c r="A2345" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2346">
       <c r="A2346" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2347">
@@ -42669,11 +42669,11 @@
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2347" t="n">
@@ -42683,19 +42683,19 @@
     <row r="2348">
       <c r="A2348" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2679</v>
+        <v>2769</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2349">
@@ -42705,11 +42705,11 @@
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2349" t="n">
@@ -42719,19 +42719,19 @@
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2351">
@@ -42741,15 +42741,15 @@
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2352">
@@ -42759,11 +42759,11 @@
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2352" t="n">
@@ -42773,37 +42773,37 @@
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2701</v>
+        <v>2817</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2354">
       <c r="A2354" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2355">
@@ -42813,11 +42813,11 @@
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2355" t="n">
@@ -42827,19 +42827,19 @@
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2357">
@@ -42849,33 +42849,33 @@
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2665</v>
+        <v>2755</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>141</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2359">
@@ -42885,15 +42885,15 @@
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2360">
@@ -42903,15 +42903,15 @@
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2361">
@@ -42921,11 +42921,11 @@
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2361" t="n">
@@ -42935,37 +42935,37 @@
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2363">
       <c r="A2363" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2364">
@@ -42975,11 +42975,11 @@
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2364" t="n">
@@ -42993,15 +42993,15 @@
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2366">
@@ -43011,11 +43011,11 @@
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - HB</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2366" t="n">
@@ -43029,15 +43029,15 @@
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2368">
@@ -43047,51 +43047,51 @@
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2369">
       <c r="A2369" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2370">
       <c r="A2370" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2371">
@@ -43101,33 +43101,33 @@
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2372">
       <c r="A2372" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2373">
@@ -43137,69 +43137,69 @@
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2374">
       <c r="A2374" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2376">
       <c r="A2376" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2819</v>
+        <v>2651</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2377">
@@ -43209,11 +43209,11 @@
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2699</v>
+        <v>2819</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2377" t="n">
@@ -43223,19 +43223,19 @@
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2706</v>
+        <v>2699</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2379">
@@ -43245,11 +43245,11 @@
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2379" t="n">
@@ -43259,127 +43259,127 @@
     <row r="2380">
       <c r="A2380" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2693</v>
+        <v>2707</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2381">
       <c r="A2381" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2383">
       <c r="A2383" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2386">
       <c r="A2386" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2387">
@@ -43389,11 +43389,11 @@
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2387" t="n">
@@ -43403,37 +43403,37 @@
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2390">
@@ -43443,15 +43443,15 @@
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2825</v>
+        <v>2773</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2391">
@@ -43461,15 +43461,15 @@
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2787</v>
+        <v>2825</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2392">
@@ -43479,33 +43479,33 @@
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2648</v>
+        <v>2787</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2394">
@@ -43515,15 +43515,15 @@
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2395">
@@ -43533,11 +43533,11 @@
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2395" t="n">
@@ -43551,33 +43551,33 @@
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2786</v>
+        <v>2780</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2398">
@@ -43587,15 +43587,15 @@
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2399">
@@ -43605,11 +43605,11 @@
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2399" t="n">
@@ -43619,19 +43619,19 @@
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2401">
@@ -43641,15 +43641,15 @@
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2402">
@@ -43659,15 +43659,15 @@
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2403">
@@ -43677,11 +43677,11 @@
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2403" t="n">
@@ -43695,11 +43695,11 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2404" t="n">
@@ -43713,11 +43713,11 @@
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2405" t="n">
@@ -43727,55 +43727,55 @@
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2409">
@@ -43785,11 +43785,11 @@
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2409" t="n">
@@ -43803,11 +43803,11 @@
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2410" t="n">
@@ -43817,19 +43817,19 @@
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2412">
@@ -43839,11 +43839,11 @@
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2412" t="n">
@@ -43857,11 +43857,11 @@
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2413" t="n">
@@ -43875,11 +43875,11 @@
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2414" t="n">
@@ -43893,15 +43893,15 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2416">
@@ -43911,15 +43911,15 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2417">
@@ -43929,11 +43929,11 @@
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2417" t="n">
@@ -43943,37 +43943,37 @@
     <row r="2418">
       <c r="A2418" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2419">
       <c r="A2419" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2420">
@@ -43983,50 +43983,68 @@
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2421">
       <c r="A2421" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2422">
       <c r="A2422" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2422" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2422" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2422" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2423">
+      <c r="A2423" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2423" t="n">
         <v>2801</v>
       </c>
-      <c r="C2422" t="inlineStr">
+      <c r="C2423" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2422" t="n">
+      <c r="D2423" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:58:59
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2423"/>
+  <dimension ref="A1:D2424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42143,37 +42143,37 @@
     <row r="2318">
       <c r="A2318" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2750</v>
+        <v>2828</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2319">
       <c r="A2319" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2320">
@@ -42183,51 +42183,51 @@
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2321">
       <c r="A2321" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2322">
       <c r="A2322" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2323">
@@ -42237,15 +42237,15 @@
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2324">
@@ -42255,11 +42255,11 @@
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>DANIELY PEREIRA PINHEIRO</t>
+          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
         </is>
       </c>
       <c r="D2324" t="n">
@@ -42269,19 +42269,19 @@
     <row r="2325">
       <c r="A2325" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY PEREIRA PINHEIRO</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2326">
@@ -42291,11 +42291,11 @@
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2326" t="n">
@@ -42309,11 +42309,11 @@
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2327" t="n">
@@ -42327,11 +42327,11 @@
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2328" t="n">
@@ -42341,73 +42341,73 @@
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2765</v>
+        <v>2820</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2741</v>
+        <v>2765</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2332">
       <c r="A2332" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2758</v>
+        <v>2741</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2332" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2333">
@@ -42417,51 +42417,51 @@
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2659</v>
+        <v>2758</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2333" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2334">
       <c r="A2334" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2669</v>
+        <v>2659</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2334" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2335" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2336">
@@ -42471,11 +42471,11 @@
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2336" t="n">
@@ -42485,19 +42485,19 @@
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2676</v>
+        <v>2673</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2338">
@@ -42507,69 +42507,69 @@
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2760</v>
+        <v>2676</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2823</v>
+        <v>2760</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>80</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2792</v>
+        <v>2823</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2341">
       <c r="A2341" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2342">
@@ -42579,15 +42579,15 @@
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2343">
@@ -42597,15 +42597,15 @@
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2344">
@@ -42615,15 +42615,15 @@
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2345">
@@ -42633,11 +42633,11 @@
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D2345" t="n">
@@ -42647,37 +42647,37 @@
     <row r="2346">
       <c r="A2346" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2347">
       <c r="A2347" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2348">
@@ -42687,11 +42687,11 @@
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2348" t="n">
@@ -42701,19 +42701,19 @@
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2679</v>
+        <v>2769</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2350">
@@ -42723,11 +42723,11 @@
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2350" t="n">
@@ -42737,19 +42737,19 @@
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2352">
@@ -42759,15 +42759,15 @@
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2353">
@@ -42777,11 +42777,11 @@
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2353" t="n">
@@ -42791,37 +42791,37 @@
     <row r="2354">
       <c r="A2354" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2701</v>
+        <v>2817</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2356">
@@ -42831,11 +42831,11 @@
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2356" t="n">
@@ -42845,19 +42845,19 @@
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2358">
@@ -42867,33 +42867,33 @@
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2359">
       <c r="A2359" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2665</v>
+        <v>2755</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>141</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2360">
@@ -42903,15 +42903,15 @@
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2361">
@@ -42921,15 +42921,15 @@
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2362">
@@ -42939,11 +42939,11 @@
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2362" t="n">
@@ -42953,37 +42953,37 @@
     <row r="2363">
       <c r="A2363" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2365">
@@ -42993,11 +42993,11 @@
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2365" t="n">
@@ -43011,15 +43011,15 @@
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2367">
@@ -43029,15 +43029,15 @@
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2368">
@@ -43047,15 +43047,15 @@
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2369">
@@ -43065,51 +43065,51 @@
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2370">
       <c r="A2370" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2372">
@@ -43119,33 +43119,33 @@
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2373">
       <c r="A2373" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2374">
@@ -43155,69 +43155,69 @@
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2376">
       <c r="A2376" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2819</v>
+        <v>2651</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2378">
@@ -43227,11 +43227,11 @@
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2699</v>
+        <v>2819</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2378" t="n">
@@ -43241,19 +43241,19 @@
     <row r="2379">
       <c r="A2379" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2706</v>
+        <v>2699</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2380">
@@ -43263,11 +43263,11 @@
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2380" t="n">
@@ -43277,127 +43277,127 @@
     <row r="2381">
       <c r="A2381" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2693</v>
+        <v>2707</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2383">
       <c r="A2383" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2386">
       <c r="A2386" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2388">
@@ -43407,11 +43407,11 @@
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2388" t="n">
@@ -43421,37 +43421,37 @@
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2391">
@@ -43461,15 +43461,15 @@
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2825</v>
+        <v>2773</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2392">
@@ -43479,15 +43479,15 @@
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2787</v>
+        <v>2825</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2393">
@@ -43497,33 +43497,33 @@
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2648</v>
+        <v>2787</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2395">
@@ -43533,15 +43533,15 @@
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2396">
@@ -43551,11 +43551,11 @@
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2396" t="n">
@@ -43569,33 +43569,33 @@
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2786</v>
+        <v>2780</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2399">
@@ -43605,15 +43605,15 @@
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2400">
@@ -43623,11 +43623,11 @@
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2400" t="n">
@@ -43637,19 +43637,19 @@
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2402">
@@ -43659,15 +43659,15 @@
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2403">
@@ -43677,15 +43677,15 @@
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2404">
@@ -43695,11 +43695,11 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2404" t="n">
@@ -43713,11 +43713,11 @@
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2405" t="n">
@@ -43731,11 +43731,11 @@
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2406" t="n">
@@ -43745,55 +43745,55 @@
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2410">
@@ -43803,11 +43803,11 @@
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2410" t="n">
@@ -43821,11 +43821,11 @@
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2411" t="n">
@@ -43835,19 +43835,19 @@
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2413">
@@ -43857,11 +43857,11 @@
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2413" t="n">
@@ -43875,11 +43875,11 @@
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2414" t="n">
@@ -43893,11 +43893,11 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2415" t="n">
@@ -43911,15 +43911,15 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2417">
@@ -43929,15 +43929,15 @@
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,11 +43947,11 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2418" t="n">
@@ -43961,37 +43961,37 @@
     <row r="2419">
       <c r="A2419" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2421">
@@ -44001,50 +44001,68 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2422">
       <c r="A2422" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2423" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2423" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2423" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2424">
+      <c r="A2424" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2424" t="n">
         <v>2801</v>
       </c>
-      <c r="C2423" t="inlineStr">
+      <c r="C2424" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2423" t="n">
+      <c r="D2424" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:00:53
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2424"/>
+  <dimension ref="A1:D2425"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>FABIOLA ALVES SILVA - HIBRIDO</t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -41279,19 +41279,19 @@
     <row r="2270">
       <c r="A2270" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2270" t="n">
-        <v>2799</v>
+        <v>2829</v>
       </c>
       <c r="C2270" t="inlineStr">
         <is>
-          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
+          <t>LAIS ANDRADE VIRIATO - FARMA</t>
         </is>
       </c>
       <c r="D2270" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2271">
@@ -41301,33 +41301,33 @@
         </is>
       </c>
       <c r="B2271" t="n">
-        <v>2719</v>
+        <v>2799</v>
       </c>
       <c r="C2271" t="inlineStr">
         <is>
-          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
+          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
         </is>
       </c>
       <c r="D2271" t="n">
-        <v>39</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2272">
       <c r="A2272" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2272" t="n">
-        <v>2731</v>
+        <v>2719</v>
       </c>
       <c r="C2272" t="inlineStr">
         <is>
-          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
+          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
         </is>
       </c>
       <c r="D2272" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2273">
@@ -41337,15 +41337,15 @@
         </is>
       </c>
       <c r="B2273" t="n">
-        <v>2732</v>
+        <v>2731</v>
       </c>
       <c r="C2273" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
+          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
         </is>
       </c>
       <c r="D2273" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2274">
@@ -41355,51 +41355,51 @@
         </is>
       </c>
       <c r="B2274" t="n">
-        <v>2733</v>
+        <v>2732</v>
       </c>
       <c r="C2274" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
+          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
         </is>
       </c>
       <c r="D2274" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2275" t="n">
-        <v>2752</v>
+        <v>2733</v>
       </c>
       <c r="C2275" t="inlineStr">
         <is>
-          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
+          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
         </is>
       </c>
       <c r="D2275" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2276">
       <c r="A2276" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2276" t="n">
-        <v>2662</v>
+        <v>2752</v>
       </c>
       <c r="C2276" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
+          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
         </is>
       </c>
       <c r="D2276" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2277">
@@ -41409,15 +41409,15 @@
         </is>
       </c>
       <c r="B2277" t="n">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="C2277" t="inlineStr">
         <is>
-          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
         </is>
       </c>
       <c r="D2277" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2278">
@@ -41427,15 +41427,15 @@
         </is>
       </c>
       <c r="B2278" t="n">
-        <v>2685</v>
+        <v>2663</v>
       </c>
       <c r="C2278" t="inlineStr">
         <is>
-          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
+          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
         </is>
       </c>
       <c r="D2278" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2279">
@@ -41445,15 +41445,15 @@
         </is>
       </c>
       <c r="B2279" t="n">
-        <v>2718</v>
+        <v>2685</v>
       </c>
       <c r="C2279" t="inlineStr">
         <is>
-          <t>KALILLA FERREIRA COSTA - FARMA</t>
+          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2279" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2280">
@@ -41463,15 +41463,15 @@
         </is>
       </c>
       <c r="B2280" t="n">
-        <v>2674</v>
+        <v>2718</v>
       </c>
       <c r="C2280" t="inlineStr">
         <is>
-          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
+          <t>KALILLA FERREIRA COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2280" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2281">
@@ -41481,15 +41481,15 @@
         </is>
       </c>
       <c r="B2281" t="n">
-        <v>2753</v>
+        <v>2674</v>
       </c>
       <c r="C2281" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA - HB</t>
+          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
         </is>
       </c>
       <c r="D2281" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2282">
@@ -41499,15 +41499,15 @@
         </is>
       </c>
       <c r="B2282" t="n">
-        <v>2772</v>
+        <v>2753</v>
       </c>
       <c r="C2282" t="inlineStr">
         <is>
-          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA - HB</t>
         </is>
       </c>
       <c r="D2282" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2283">
@@ -41517,51 +41517,51 @@
         </is>
       </c>
       <c r="B2283" t="n">
-        <v>2827</v>
+        <v>2772</v>
       </c>
       <c r="C2283" t="inlineStr">
         <is>
-          <t>JOELTON MUNIZ DE SOUZA - HB</t>
+          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2283" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2284">
       <c r="A2284" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2284" t="n">
-        <v>2756</v>
+        <v>2827</v>
       </c>
       <c r="C2284" t="inlineStr">
         <is>
-          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
+          <t>JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2284" t="n">
-        <v>39</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2285">
       <c r="A2285" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2285" t="n">
-        <v>2813</v>
+        <v>2756</v>
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
+          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
         </is>
       </c>
       <c r="D2285" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2286">
@@ -41571,15 +41571,15 @@
         </is>
       </c>
       <c r="B2286" t="n">
-        <v>2738</v>
+        <v>2813</v>
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
+          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="D2286" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2287">
@@ -41589,11 +41589,11 @@
         </is>
       </c>
       <c r="B2287" t="n">
-        <v>2739</v>
+        <v>2738</v>
       </c>
       <c r="C2287" t="inlineStr">
         <is>
-          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
+          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2287" t="n">
@@ -41607,33 +41607,33 @@
         </is>
       </c>
       <c r="B2288" t="n">
-        <v>2824</v>
+        <v>2739</v>
       </c>
       <c r="C2288" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2288" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2289">
       <c r="A2289" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2289" t="n">
-        <v>2747</v>
+        <v>2824</v>
       </c>
       <c r="C2289" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2289" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2290">
@@ -41643,11 +41643,11 @@
         </is>
       </c>
       <c r="B2290" t="n">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="C2290" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2290" t="n">
@@ -41657,73 +41657,73 @@
     <row r="2291">
       <c r="A2291" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2291" t="n">
-        <v>2766</v>
+        <v>2748</v>
       </c>
       <c r="C2291" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2291" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2292">
       <c r="A2292" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2767</v>
+        <v>2766</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2292" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2293">
       <c r="A2293" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2688</v>
+        <v>2767</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2293" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2294">
       <c r="A2294" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2694</v>
+        <v>2688</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2294" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2295">
@@ -41733,15 +41733,15 @@
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2714</v>
+        <v>2694</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2295" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2296">
@@ -41751,15 +41751,15 @@
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2722</v>
+        <v>2714</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2296" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2297">
@@ -41769,15 +41769,15 @@
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2298">
@@ -41787,15 +41787,15 @@
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2803</v>
+        <v>2723</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2298" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2299">
@@ -41805,11 +41805,11 @@
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2804</v>
+        <v>2803</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2299" t="n">
@@ -41819,55 +41819,55 @@
     <row r="2300">
       <c r="A2300" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2647</v>
+        <v>2804</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>147</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2301">
       <c r="A2301" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2661</v>
+        <v>2647</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>76</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2302">
       <c r="A2302" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2686</v>
+        <v>2661</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2302" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2303">
@@ -41877,11 +41877,11 @@
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2303" t="n">
@@ -41891,109 +41891,109 @@
     <row r="2304">
       <c r="A2304" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2681</v>
+        <v>2687</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2304" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2305" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2826</v>
+        <v>2682</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2677</v>
+        <v>2826</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2309">
       <c r="A2309" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2735</v>
+        <v>2678</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2309" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2310">
@@ -42003,15 +42003,15 @@
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2311">
@@ -42021,15 +42021,15 @@
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2312">
@@ -42039,15 +42039,15 @@
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2743</v>
+        <v>2737</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2313">
@@ -42057,11 +42057,11 @@
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2313" t="n">
@@ -42075,15 +42075,15 @@
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2315">
@@ -42093,105 +42093,105 @@
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2783</v>
+        <v>2745</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2316">
       <c r="A2316" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2768</v>
+        <v>2783</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2317">
       <c r="A2317" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2318">
       <c r="A2318" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2828</v>
+        <v>2703</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2319">
       <c r="A2319" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2750</v>
+        <v>2828</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2320">
       <c r="A2320" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2321">
@@ -42201,51 +42201,51 @@
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2322">
       <c r="A2322" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2323">
       <c r="A2323" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2324">
@@ -42255,15 +42255,15 @@
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2325">
@@ -42273,11 +42273,11 @@
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>DANIELY PEREIRA PINHEIRO</t>
+          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
         </is>
       </c>
       <c r="D2325" t="n">
@@ -42287,19 +42287,19 @@
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY PEREIRA PINHEIRO</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2327">
@@ -42309,11 +42309,11 @@
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2327" t="n">
@@ -42327,11 +42327,11 @@
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2328" t="n">
@@ -42345,11 +42345,11 @@
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2329" t="n">
@@ -42359,73 +42359,73 @@
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2765</v>
+        <v>2820</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2332">
       <c r="A2332" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2741</v>
+        <v>2765</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2332" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2333">
       <c r="A2333" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2758</v>
+        <v>2741</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2333" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2334">
@@ -42435,51 +42435,51 @@
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2659</v>
+        <v>2758</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2334" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2669</v>
+        <v>2659</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2335" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2336">
       <c r="A2336" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2336" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2337">
@@ -42489,11 +42489,11 @@
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2337" t="n">
@@ -42503,19 +42503,19 @@
     <row r="2338">
       <c r="A2338" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2676</v>
+        <v>2673</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2339">
@@ -42525,69 +42525,69 @@
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2760</v>
+        <v>2676</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2823</v>
+        <v>2760</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>80</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2341">
       <c r="A2341" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2792</v>
+        <v>2823</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2343">
@@ -42597,15 +42597,15 @@
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2344">
@@ -42615,15 +42615,15 @@
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2345">
@@ -42633,15 +42633,15 @@
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2346">
@@ -42651,11 +42651,11 @@
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D2346" t="n">
@@ -42665,37 +42665,37 @@
     <row r="2347">
       <c r="A2347" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2348">
       <c r="A2348" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2349">
@@ -42705,11 +42705,11 @@
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2349" t="n">
@@ -42719,19 +42719,19 @@
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2679</v>
+        <v>2769</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2351">
@@ -42741,11 +42741,11 @@
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2351" t="n">
@@ -42755,19 +42755,19 @@
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2353">
@@ -42777,15 +42777,15 @@
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2354">
@@ -42795,11 +42795,11 @@
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2354" t="n">
@@ -42809,37 +42809,37 @@
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2701</v>
+        <v>2817</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2357">
@@ -42849,11 +42849,11 @@
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2357" t="n">
@@ -42863,19 +42863,19 @@
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2359">
@@ -42885,33 +42885,33 @@
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2360">
       <c r="A2360" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2665</v>
+        <v>2755</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>141</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2361">
@@ -42921,15 +42921,15 @@
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2362">
@@ -42939,15 +42939,15 @@
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2363">
@@ -42957,11 +42957,11 @@
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2363" t="n">
@@ -42971,37 +42971,37 @@
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2365">
       <c r="A2365" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2366">
@@ -43011,11 +43011,11 @@
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2366" t="n">
@@ -43029,15 +43029,15 @@
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2368">
@@ -43047,15 +43047,15 @@
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2369">
@@ -43065,15 +43065,15 @@
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2370">
@@ -43083,51 +43083,51 @@
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2372">
       <c r="A2372" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2373">
@@ -43137,33 +43137,33 @@
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2374">
       <c r="A2374" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2375">
@@ -43173,69 +43173,69 @@
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2376">
       <c r="A2376" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2819</v>
+        <v>2651</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2379">
@@ -43245,11 +43245,11 @@
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2699</v>
+        <v>2819</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2379" t="n">
@@ -43259,19 +43259,19 @@
     <row r="2380">
       <c r="A2380" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2706</v>
+        <v>2699</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2381">
@@ -43281,11 +43281,11 @@
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2381" t="n">
@@ -43295,127 +43295,127 @@
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2693</v>
+        <v>2707</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2383">
       <c r="A2383" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2386">
       <c r="A2386" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2389">
@@ -43425,11 +43425,11 @@
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2389" t="n">
@@ -43439,37 +43439,37 @@
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2392">
@@ -43479,15 +43479,15 @@
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2825</v>
+        <v>2773</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2393">
@@ -43497,15 +43497,15 @@
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2787</v>
+        <v>2825</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2394">
@@ -43515,33 +43515,33 @@
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2648</v>
+        <v>2787</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2396">
@@ -43551,15 +43551,15 @@
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2397">
@@ -43569,11 +43569,11 @@
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2397" t="n">
@@ -43587,33 +43587,33 @@
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2786</v>
+        <v>2780</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2400">
@@ -43623,15 +43623,15 @@
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2401">
@@ -43641,11 +43641,11 @@
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2401" t="n">
@@ -43655,19 +43655,19 @@
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2403">
@@ -43677,15 +43677,15 @@
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2404">
@@ -43695,15 +43695,15 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2405">
@@ -43713,11 +43713,11 @@
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2405" t="n">
@@ -43731,11 +43731,11 @@
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2406" t="n">
@@ -43749,11 +43749,11 @@
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2407" t="n">
@@ -43763,55 +43763,55 @@
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2411">
@@ -43821,11 +43821,11 @@
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2411" t="n">
@@ -43839,11 +43839,11 @@
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2412" t="n">
@@ -43853,19 +43853,19 @@
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2414">
@@ -43875,11 +43875,11 @@
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2414" t="n">
@@ -43893,11 +43893,11 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2415" t="n">
@@ -43911,11 +43911,11 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2416" t="n">
@@ -43929,15 +43929,15 @@
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,15 +43947,15 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2419">
@@ -43965,11 +43965,11 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2419" t="n">
@@ -43979,37 +43979,37 @@
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2421">
       <c r="A2421" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2422">
@@ -44019,50 +44019,68 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2424">
       <c r="A2424" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2424" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2424" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2424" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2425">
+      <c r="A2425" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2425" t="n">
         <v>2801</v>
       </c>
-      <c r="C2424" t="inlineStr">
+      <c r="C2425" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2424" t="n">
+      <c r="D2425" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:00:58
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -1173,7 +1173,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -25672,7 +25672,7 @@
     <row r="1403">
       <c r="A1403" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B1403" t="n">
@@ -25690,7 +25690,7 @@
     <row r="1404">
       <c r="A1404" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B1404" t="n">
@@ -25708,7 +25708,7 @@
     <row r="1405">
       <c r="A1405" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B1405" t="n">
@@ -25726,7 +25726,7 @@
     <row r="1406">
       <c r="A1406" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B1406" t="n">
@@ -25744,7 +25744,7 @@
     <row r="1407">
       <c r="A1407" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B1407" t="n">
@@ -25762,7 +25762,7 @@
     <row r="1408">
       <c r="A1408" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B1408" t="n">
@@ -27814,7 +27814,7 @@
     <row r="1522">
       <c r="A1522" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B1522" t="n">
@@ -27832,7 +27832,7 @@
     <row r="1523">
       <c r="A1523" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B1523" t="n">
@@ -42827,7 +42827,7 @@
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2356" t="n">
@@ -42845,7 +42845,7 @@
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2357" t="n">

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:01
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2424"/>
+  <dimension ref="A1:D2426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17896,7 +17896,7 @@
     <row r="971">
       <c r="A971" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B971" t="n">
@@ -23142,7 +23142,7 @@
       </c>
       <c r="C1262" t="inlineStr">
         <is>
-          <t>JOÃO MARCOS DE SOUZA FERREIRA - HIBRIDO</t>
+          <t>INATIVO- JOÃO MARCOS DE SOUZA FERREIRA</t>
         </is>
       </c>
       <c r="D1262" t="n">
@@ -27202,7 +27202,7 @@
     <row r="1488">
       <c r="A1488" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B1488" t="n">
@@ -27238,7 +27238,7 @@
     <row r="1490">
       <c r="A1490" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B1490" t="n">
@@ -33412,7 +33412,7 @@
     <row r="1833">
       <c r="A1833" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B1833" t="n">
@@ -35375,7 +35375,7 @@
     <row r="1942">
       <c r="A1942" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B1942" t="n">
@@ -36815,7 +36815,7 @@
     <row r="2022">
       <c r="A2022" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2022" t="n">
@@ -39047,7 +39047,7 @@
     <row r="2146">
       <c r="A2146" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2146" t="n">
@@ -40037,7 +40037,7 @@
     <row r="2201">
       <c r="A2201" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2201" t="n">
@@ -41819,199 +41819,199 @@
     <row r="2300">
       <c r="A2300" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2647</v>
+        <v>2830</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>SETOR VAGO BALSAS 1</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2301">
       <c r="A2301" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2661</v>
+        <v>2831</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>SETOR VAGO BALSAS 2</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>76</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2302">
       <c r="A2302" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2686</v>
+        <v>2647</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2302" t="n">
-        <v>120</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2303">
       <c r="A2303" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2687</v>
+        <v>2661</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2303" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2304">
       <c r="A2304" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2681</v>
+        <v>2686</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2304" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2682</v>
+        <v>2687</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2305" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2826</v>
+        <v>2681</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2677</v>
+        <v>2682</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>72</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2678</v>
+        <v>2826</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2309">
       <c r="A2309" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2735</v>
+        <v>2677</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2309" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2310">
       <c r="A2310" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2736</v>
+        <v>2678</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2311">
@@ -42021,11 +42021,11 @@
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2737</v>
+        <v>2735</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2311" t="n">
@@ -42039,11 +42039,11 @@
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2743</v>
+        <v>2736</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2312" t="n">
@@ -42057,15 +42057,15 @@
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2744</v>
+        <v>2737</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2314">
@@ -42075,15 +42075,15 @@
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2745</v>
+        <v>2743</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2315">
@@ -42093,11 +42093,11 @@
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2783</v>
+        <v>2744</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2315" t="n">
@@ -42107,19 +42107,19 @@
     <row r="2316">
       <c r="A2316" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2768</v>
+        <v>2745</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>69</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2317">
@@ -42129,15 +42129,15 @@
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2703</v>
+        <v>2783</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2318">
@@ -42147,15 +42147,15 @@
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2828</v>
+        <v>2768</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2319">
@@ -42165,69 +42165,69 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2750</v>
+        <v>2703</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2320">
       <c r="A2320" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2689</v>
+        <v>2828</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2321">
       <c r="A2321" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2708</v>
+        <v>2750</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2322">
       <c r="A2322" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2709</v>
+        <v>2689</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>39</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2323">
@@ -42237,11 +42237,11 @@
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2789</v>
+        <v>2708</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2323" t="n">
@@ -42251,19 +42251,19 @@
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2790</v>
+        <v>2709</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>114</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2325">
@@ -42273,65 +42273,65 @@
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2791</v>
+        <v>2789</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>DANIELY PEREIRA PINHEIRO</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2805</v>
+        <v>2790</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2806</v>
+        <v>2791</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>DANIELY PEREIRA PINHEIRO</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2328">
       <c r="A2328" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2807</v>
+        <v>2805</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2328" t="n">
@@ -42341,15 +42341,15 @@
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2808</v>
+        <v>2806</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2329" t="n">
@@ -42359,37 +42359,37 @@
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2820</v>
+        <v>2807</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2765</v>
+        <v>2808</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2332">
@@ -42399,15 +42399,15 @@
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2741</v>
+        <v>2820</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2332" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2333">
@@ -42417,51 +42417,51 @@
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2758</v>
+        <v>2765</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2333" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2334">
       <c r="A2334" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2659</v>
+        <v>2741</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2334" t="n">
-        <v>100</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2669</v>
+        <v>2758</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2335" t="n">
-        <v>135</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2336">
@@ -42471,141 +42471,141 @@
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2672</v>
+        <v>2659</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2336" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2673</v>
+        <v>2669</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2338">
       <c r="A2338" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2676</v>
+        <v>2672</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2760</v>
+        <v>2673</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2823</v>
+        <v>2676</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2341">
       <c r="A2341" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2792</v>
+        <v>2760</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2793</v>
+        <v>2823</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2343">
       <c r="A2343" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2802</v>
+        <v>2792</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2344">
@@ -42615,11 +42615,11 @@
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2656</v>
+        <v>2793</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2344" t="n">
@@ -42633,15 +42633,15 @@
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2657</v>
+        <v>2802</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2346">
@@ -42651,33 +42651,33 @@
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2658</v>
+        <v>2656</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2347">
       <c r="A2347" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2729</v>
+        <v>2657</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2348">
@@ -42687,105 +42687,105 @@
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2759</v>
+        <v>2658</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2769</v>
+        <v>2729</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2679</v>
+        <v>2759</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2680</v>
+        <v>2769</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2815</v>
+        <v>2679</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2816</v>
+        <v>2680</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2354">
@@ -42795,87 +42795,87 @@
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2817</v>
+        <v>2815</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2701</v>
+        <v>2816</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2644</v>
+        <v>2817</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2645</v>
+        <v>2701</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2754</v>
+        <v>2644</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2359">
@@ -42885,51 +42885,51 @@
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2755</v>
+        <v>2645</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>80</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2360">
       <c r="A2360" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2665</v>
+        <v>2754</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>141</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2361">
       <c r="A2361" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2667</v>
+        <v>2755</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2362">
@@ -42939,15 +42939,15 @@
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2727</v>
+        <v>2665</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>120</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2363">
@@ -42957,69 +42957,69 @@
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2728</v>
+        <v>2667</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2814</v>
+        <v>2727</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2365">
       <c r="A2365" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2646</v>
+        <v>2728</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2650</v>
+        <v>2814</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2367">
@@ -43029,15 +43029,15 @@
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2652</v>
+        <v>2646</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2368">
@@ -43047,11 +43047,11 @@
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2653</v>
+        <v>2650</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2368" t="n">
@@ -43065,15 +43065,15 @@
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2654</v>
+        <v>2652</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2370">
@@ -43083,33 +43083,33 @@
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2655</v>
+        <v>2653</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2821</v>
+        <v>2654</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2372">
@@ -43119,87 +43119,87 @@
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2683</v>
+        <v>2655</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2373">
       <c r="A2373" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2684</v>
+        <v>2821</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2374">
       <c r="A2374" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2749</v>
+        <v>2683</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>111</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2812</v>
+        <v>2684</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>145</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2376">
       <c r="A2376" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2715</v>
+        <v>2749</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2377">
@@ -43209,11 +43209,11 @@
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2651</v>
+        <v>2812</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2377" t="n">
@@ -43223,145 +43223,145 @@
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2819</v>
+        <v>2715</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2379">
       <c r="A2379" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2699</v>
+        <v>2651</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2380">
       <c r="A2380" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2706</v>
+        <v>2819</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2381">
       <c r="A2381" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2707</v>
+        <v>2699</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2693</v>
+        <v>2706</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2383">
       <c r="A2383" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2705</v>
+        <v>2707</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>146</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2664</v>
+        <v>2693</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2670</v>
+        <v>2705</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>69</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2386">
@@ -43371,141 +43371,141 @@
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2730</v>
+        <v>2664</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2691</v>
+        <v>2730</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2692</v>
+        <v>2671</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2724</v>
+        <v>2691</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2773</v>
+        <v>2692</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2825</v>
+        <v>2724</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2787</v>
+        <v>2773</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2394">
@@ -43515,51 +43515,51 @@
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2648</v>
+        <v>2825</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2666</v>
+        <v>2787</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>63</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2779</v>
+        <v>2648</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2397">
@@ -43569,15 +43569,15 @@
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2780</v>
+        <v>2666</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2398">
@@ -43587,51 +43587,51 @@
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2786</v>
+        <v>2779</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2660</v>
+        <v>2780</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2716</v>
+        <v>2786</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2401">
@@ -43641,51 +43641,51 @@
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2734</v>
+        <v>2660</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2742</v>
+        <v>2716</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2794</v>
+        <v>2734</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2404">
@@ -43695,11 +43695,11 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2795</v>
+        <v>2742</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2404" t="n">
@@ -43713,15 +43713,15 @@
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2796</v>
+        <v>2794</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2406">
@@ -43731,11 +43731,11 @@
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2797</v>
+        <v>2795</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2406" t="n">
@@ -43749,11 +43749,11 @@
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2798</v>
+        <v>2796</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2407" t="n">
@@ -43763,73 +43763,73 @@
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2668</v>
+        <v>2797</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2690</v>
+        <v>2798</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2696</v>
+        <v>2668</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2697</v>
+        <v>2690</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2412">
@@ -43839,11 +43839,11 @@
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2698</v>
+        <v>2696</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2412" t="n">
@@ -43853,37 +43853,37 @@
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2775</v>
+        <v>2697</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2776</v>
+        <v>2698</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2415">
@@ -43893,11 +43893,11 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2777</v>
+        <v>2775</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2415" t="n">
@@ -43911,11 +43911,11 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2778</v>
+        <v>2776</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2416" t="n">
@@ -43929,15 +43929,15 @@
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2781</v>
+        <v>2777</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,11 +43947,11 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2822</v>
+        <v>2778</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2418" t="n">
@@ -43965,33 +43965,33 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2740</v>
+        <v>2781</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2710</v>
+        <v>2822</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2421">
@@ -44001,51 +44001,51 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2711</v>
+        <v>2740</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2422">
       <c r="A2422" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2717</v>
+        <v>2711</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2424">
@@ -44055,14 +44055,50 @@
         </is>
       </c>
       <c r="B2424" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2424" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2424" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2425">
+      <c r="A2425" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2425" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2425" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2425" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2426">
+      <c r="A2426" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2426" t="n">
         <v>2801</v>
       </c>
-      <c r="C2424" t="inlineStr">
+      <c r="C2426" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2424" t="n">
+      <c r="D2426" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>